<commit_message>
The baseline's own equipment keeps its inventory age in later stages, so the boiler's sunk cost is priced
Stage 0 charges everything it carries, and the ageing merge dated that equipment to the simulation
year and marked it replaced by nothing, so a 2010 boiler counted as new and its sunk cost was never
written off when the heat pump replaced it. Only stages 1.. put anything into the building now. The
synthetic inventory boiler and the worked examples' register carry a like-for-like price override,
because the test database has no device rows; the two multi-stage worked examples are regenerated,
still unreviewed: the kept boiler is now re-purchased in year 8 and earns its own write-down.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/worked_examples/staged/three_stages_with_loans_and_a_staged_grant.xlsx
+++ b/tests/worked_examples/staged/three_stages_with_loans_and_a_staged_grant.xlsx
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>60648.43755924105</v>
+        <v>64641.02342882127</v>
       </c>
       <c r="C44" t="n">
         <v>0.01</v>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>4076.527645188313</v>
+        <v>4344.892129553368</v>
       </c>
       <c r="C45" t="n">
         <v>0.01</v>
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>15147.69682898998</v>
+        <v>19140.2826985702</v>
       </c>
       <c r="C47" t="n">
         <v>0.01</v>

</xml_diff>